<commit_message>
Update species name resolging
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_species_seeded.xlsx
+++ b/data/raw/data_raw_species_seeded.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marku\Documents\GitHub\2025_greeen_prairie\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA07FC5E-D564-4520-9B6F-9A51D4A14621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF69013-4511-40F8-90CE-7C6C71C890E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -254,24 +254,12 @@
     <t>ASCTUB</t>
   </si>
   <si>
-    <t>ASTERI</t>
-  </si>
-  <si>
-    <t>ASTLAE</t>
-  </si>
-  <si>
     <t>ASTOOL</t>
   </si>
   <si>
-    <t>ASTSAG</t>
-  </si>
-  <si>
     <t>BAPLAC</t>
   </si>
   <si>
-    <t>CASFAS</t>
-  </si>
-  <si>
     <t>CORLAN</t>
   </si>
   <si>
@@ -311,9 +299,6 @@
     <t>PENHIR</t>
   </si>
   <si>
-    <t>PETPUR</t>
-  </si>
-  <si>
     <t>DRYARG</t>
   </si>
   <si>
@@ -345,6 +330,21 @@
   </si>
   <si>
     <t>SOLJUN</t>
+  </si>
+  <si>
+    <t>CHAFAS</t>
+  </si>
+  <si>
+    <t>DALPUR</t>
+  </si>
+  <si>
+    <t>SYMERI</t>
+  </si>
+  <si>
+    <t>SYMLAE</t>
+  </si>
+  <si>
+    <t>SYMUND</t>
   </si>
 </sst>
 </file>
@@ -625,16 +625,31 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -659,21 +674,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1009,97 +1009,97 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" s="3"/>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="45" t="s">
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
+      <c r="W1" s="51"/>
+      <c r="X1" s="51"/>
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
       <c r="AA1" s="3"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50" t="s">
+      <c r="C2" s="40" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50" t="s">
+      <c r="F2" s="40"/>
+      <c r="G2" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50" t="s">
+      <c r="H2" s="40"/>
+      <c r="I2" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="51"/>
-      <c r="K2" s="47" t="s">
+      <c r="J2" s="41"/>
+      <c r="K2" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="L2" s="37" t="s">
+      <c r="L2" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="39" t="s">
+      <c r="M2" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="40"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="39" t="s">
+      <c r="N2" s="45"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="39" t="s">
+      <c r="Q2" s="45"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="T2" s="40"/>
-      <c r="U2" s="41"/>
-      <c r="V2" s="39" t="s">
+      <c r="T2" s="45"/>
+      <c r="U2" s="46"/>
+      <c r="V2" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="W2" s="40"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="35" t="s">
+      <c r="W2" s="45"/>
+      <c r="X2" s="46"/>
+      <c r="Y2" s="42" t="s">
         <v>54</v>
       </c>
       <c r="Z2" s="22"/>
-      <c r="AA2" s="37" t="s">
+      <c r="AA2" s="39" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="60.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="38"/>
-      <c r="B3" s="48"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="4" t="s">
         <v>5</v>
       </c>
@@ -1124,8 +1124,8 @@
       <c r="J3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="48"/>
-      <c r="L3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="36"/>
       <c r="M3" s="6" t="s">
         <v>40</v>
       </c>
@@ -1162,11 +1162,11 @@
       <c r="X3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="Y3" s="36"/>
+      <c r="Y3" s="43"/>
       <c r="Z3" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="AA3" s="38"/>
+      <c r="AA3" s="36"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4160,13 +4160,6 @@
     <sortCondition ref="A3:A35"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
     <mergeCell ref="Y2:Y3"/>
     <mergeCell ref="AA2:AA3"/>
     <mergeCell ref="S2:U2"/>
@@ -4176,6 +4169,13 @@
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="M2:O2"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:AA36">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
@@ -4250,7 +4250,7 @@
     </row>
     <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="33" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="B4" s="34">
         <v>0.29972762003658182</v>
@@ -4267,7 +4267,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="B5" s="34">
         <v>0.2872234798388667</v>
@@ -4284,7 +4284,7 @@
     </row>
     <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B6" s="34">
         <v>0.48227660785515125</v>
@@ -4301,7 +4301,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="B7" s="34">
         <v>0.32078894883401449</v>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B8" s="34">
         <v>0.26028252198742302</v>
@@ -4335,7 +4335,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="B9" s="34">
         <v>0.27140262547314181</v>
@@ -4352,7 +4352,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B10" s="34">
         <v>0.27016492127382641</v>
@@ -4369,7 +4369,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B11" s="34">
         <v>0.27497679649081486</v>
@@ -4386,7 +4386,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B12" s="34">
         <v>0.27033694605655412</v>
@@ -4403,7 +4403,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B13" s="34">
         <v>0.39004517572973652</v>
@@ -4420,7 +4420,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B14" s="34">
         <v>0.27414819658748479</v>
@@ -4437,7 +4437,7 @@
     </row>
     <row r="15" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="33" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B15" s="34">
         <v>0.26615662341353147</v>
@@ -4454,7 +4454,7 @@
     </row>
     <row r="16" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="33" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B16" s="34">
         <v>0.28357843066802951</v>
@@ -4471,7 +4471,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B17" s="34">
         <v>0.41746723085724502</v>
@@ -4488,7 +4488,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B18" s="34">
         <v>0.26264409142085876</v>
@@ -4505,7 +4505,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B19" s="34">
         <v>0.2686264940093756</v>
@@ -4522,7 +4522,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B20" s="34">
         <v>0.27131590613387041</v>
@@ -4539,7 +4539,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B21" s="34">
         <v>0.27154728096054886</v>
@@ -4556,7 +4556,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B22" s="34">
         <v>0.35752772528995214</v>
@@ -4573,7 +4573,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="B23" s="34">
         <v>0.27701011773498363</v>
@@ -4590,7 +4590,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B24" s="34">
         <v>0.27740226970389947</v>
@@ -4607,7 +4607,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B25" s="34">
         <v>0.26294230415884695</v>
@@ -4624,7 +4624,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B26" s="34">
         <v>0.29586353573645868</v>
@@ -4641,7 +4641,7 @@
     </row>
     <row r="27" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="33" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B27" s="34">
         <v>0.2820087504362791</v>
@@ -4658,7 +4658,7 @@
     </row>
     <row r="28" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="33" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B28" s="34">
         <v>0.27682949822765801</v>
@@ -4675,7 +4675,7 @@
     </row>
     <row r="29" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="33" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B29" s="34">
         <v>0.3382981464396958</v>
@@ -4692,7 +4692,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B30" s="34">
         <v>0.34771840604571513</v>
@@ -4709,7 +4709,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B31" s="34">
         <v>0.34466040355715183</v>
@@ -4726,7 +4726,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B32" s="34">
         <v>0.28014792067424493</v>
@@ -4743,7 +4743,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B33" s="34">
         <v>0.2691942346709193</v>
@@ -4760,7 +4760,7 @@
     </row>
     <row r="34" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="33" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B34" s="34">
         <v>0.28008631585386579</v>

</xml_diff>

<commit_message>
Inlcude traits from Chad Zirbel
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_species_seeded.xlsx
+++ b/data/raw/data_raw_species_seeded.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marku\Documents\GitHub\2025_greeen_prairie\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68390D4E-46D8-4D19-8A3F-776E9B42B36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20512ED0-6F95-4206-892F-0B2D03D303B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="300" yWindow="0" windowWidth="18900" windowHeight="10080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculations" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="109">
   <si>
     <t>FULL DIV</t>
   </si>
@@ -345,6 +345,24 @@
   </si>
   <si>
     <t>seeded_pool_6</t>
+  </si>
+  <si>
+    <t>Androgpogon gerardii</t>
+  </si>
+  <si>
+    <t>Bouteloua curtipendula</t>
+  </si>
+  <si>
+    <t>Schizachyrium scoparium</t>
+  </si>
+  <si>
+    <t>Sporobolus cryptandrus</t>
+  </si>
+  <si>
+    <t>Panicum virgatum</t>
+  </si>
+  <si>
+    <t>Sorgasthrum nutans</t>
   </si>
 </sst>
 </file>
@@ -625,16 +643,31 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -659,21 +692,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1009,97 +1027,97 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" s="3"/>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="45" t="s">
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
+      <c r="W1" s="51"/>
+      <c r="X1" s="51"/>
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
       <c r="AA1" s="3"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50" t="s">
+      <c r="C2" s="40" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50" t="s">
+      <c r="F2" s="40"/>
+      <c r="G2" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50" t="s">
+      <c r="H2" s="40"/>
+      <c r="I2" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="51"/>
-      <c r="K2" s="47" t="s">
+      <c r="J2" s="41"/>
+      <c r="K2" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="L2" s="37" t="s">
+      <c r="L2" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="39" t="s">
+      <c r="M2" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="40"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="39" t="s">
+      <c r="N2" s="45"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="39" t="s">
+      <c r="Q2" s="45"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="T2" s="40"/>
-      <c r="U2" s="41"/>
-      <c r="V2" s="39" t="s">
+      <c r="T2" s="45"/>
+      <c r="U2" s="46"/>
+      <c r="V2" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="W2" s="40"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="35" t="s">
+      <c r="W2" s="45"/>
+      <c r="X2" s="46"/>
+      <c r="Y2" s="42" t="s">
         <v>54</v>
       </c>
       <c r="Z2" s="22"/>
-      <c r="AA2" s="37" t="s">
+      <c r="AA2" s="39" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="60.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="38"/>
-      <c r="B3" s="48"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="4" t="s">
         <v>5</v>
       </c>
@@ -1124,8 +1142,8 @@
       <c r="J3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="48"/>
-      <c r="L3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="36"/>
       <c r="M3" s="6" t="s">
         <v>40</v>
       </c>
@@ -1162,11 +1180,11 @@
       <c r="X3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="Y3" s="36"/>
+      <c r="Y3" s="43"/>
       <c r="Z3" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="AA3" s="38"/>
+      <c r="AA3" s="36"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4160,13 +4178,6 @@
     <sortCondition ref="A3:A35"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
     <mergeCell ref="Y2:Y3"/>
     <mergeCell ref="AA2:AA3"/>
     <mergeCell ref="S2:U2"/>
@@ -4176,6 +4187,13 @@
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="M2:O2"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:AA36">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
@@ -4189,7 +4207,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.54296875" bestFit="1" customWidth="1"/>
@@ -4775,11 +4793,113 @@
         <v>0</v>
       </c>
     </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="34">
+        <v>1</v>
+      </c>
+      <c r="C35" s="34">
+        <v>1</v>
+      </c>
+      <c r="D35" s="34">
+        <v>1</v>
+      </c>
+      <c r="E35" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B36" s="34">
+        <v>1</v>
+      </c>
+      <c r="C36" s="34">
+        <v>1</v>
+      </c>
+      <c r="D36" s="34">
+        <v>1</v>
+      </c>
+      <c r="E36" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B37" s="34">
+        <v>1</v>
+      </c>
+      <c r="C37" s="34">
+        <v>1</v>
+      </c>
+      <c r="D37" s="34">
+        <v>1</v>
+      </c>
+      <c r="E37" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="34">
+        <v>1</v>
+      </c>
+      <c r="C38" s="34">
+        <v>1</v>
+      </c>
+      <c r="D38" s="34">
+        <v>1</v>
+      </c>
+      <c r="E38" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="34">
+        <v>1</v>
+      </c>
+      <c r="C39" s="34">
+        <v>1</v>
+      </c>
+      <c r="D39" s="34">
+        <v>1</v>
+      </c>
+      <c r="E39" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40" s="34">
+        <v>1</v>
+      </c>
+      <c r="C40" s="34">
+        <v>1</v>
+      </c>
+      <c r="D40" s="34">
+        <v>1</v>
+      </c>
+      <c r="E40" s="34">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H34">
     <sortCondition ref="A2:A34"/>
   </sortState>
-  <conditionalFormatting sqref="B2:E34">
+  <conditionalFormatting sqref="B2:E40">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update summarize duplicates of traits matrix
Reason: Symphyotrichum oolentangiense was not in species pool in processed data
</commit_message>
<xml_diff>
--- a/data/raw/data_raw_species_seeded.xlsx
+++ b/data/raw/data_raw_species_seeded.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marku\Documents\GitHub\2025_greeen_prairie\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213C7EB7-A291-402A-877D-1A34AD2C0543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2AD2EA0-3522-416F-8BB9-263A031984B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="-90" windowWidth="18900" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculations" sheetId="1" r:id="rId1"/>
@@ -344,9 +344,6 @@
     <t>seeded_pool_6</t>
   </si>
   <si>
-    <t>Androgpogon gerardii</t>
-  </si>
-  <si>
     <t>Bouteloua curtipendula</t>
   </si>
   <si>
@@ -359,10 +356,13 @@
     <t>Panicum virgatum</t>
   </si>
   <si>
-    <t>Sorgasthrum nutans</t>
-  </si>
-  <si>
     <t>SYMURO</t>
+  </si>
+  <si>
+    <t>Andropogon gerardii</t>
+  </si>
+  <si>
+    <t>Sorghastrum nutans</t>
   </si>
 </sst>
 </file>
@@ -643,16 +643,31 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -677,21 +692,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1015,109 +1015,109 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
-    <col min="2" max="2" width="9.1796875" style="2"/>
-    <col min="11" max="12" width="9.1796875"/>
-    <col min="14" max="14" width="14.81640625" customWidth="1"/>
-    <col min="17" max="17" width="13.26953125" customWidth="1"/>
-    <col min="26" max="26" width="9.1796875"/>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="2"/>
+    <col min="11" max="12" width="9.140625"/>
+    <col min="14" max="14" width="14.85546875" customWidth="1"/>
+    <col min="17" max="17" width="13.28515625" customWidth="1"/>
+    <col min="26" max="26" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="45" t="s">
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
+      <c r="W1" s="51"/>
+      <c r="X1" s="51"/>
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
       <c r="AA1" s="3"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50" t="s">
+      <c r="C2" s="40" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50" t="s">
+      <c r="F2" s="40"/>
+      <c r="G2" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50" t="s">
+      <c r="H2" s="40"/>
+      <c r="I2" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="51"/>
-      <c r="K2" s="47" t="s">
+      <c r="J2" s="41"/>
+      <c r="K2" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="L2" s="37" t="s">
+      <c r="L2" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="39" t="s">
+      <c r="M2" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="40"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="39" t="s">
+      <c r="N2" s="45"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="39" t="s">
+      <c r="Q2" s="45"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="T2" s="40"/>
-      <c r="U2" s="41"/>
-      <c r="V2" s="39" t="s">
+      <c r="T2" s="45"/>
+      <c r="U2" s="46"/>
+      <c r="V2" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="W2" s="40"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="35" t="s">
+      <c r="W2" s="45"/>
+      <c r="X2" s="46"/>
+      <c r="Y2" s="42" t="s">
         <v>54</v>
       </c>
       <c r="Z2" s="22"/>
-      <c r="AA2" s="37" t="s">
+      <c r="AA2" s="39" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="60.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="38"/>
-      <c r="B3" s="48"/>
+    <row r="3" spans="1:27" ht="84.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="36"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="4" t="s">
         <v>5</v>
       </c>
@@ -1142,8 +1142,8 @@
       <c r="J3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="48"/>
-      <c r="L3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="36"/>
       <c r="M3" s="6" t="s">
         <v>40</v>
       </c>
@@ -1180,13 +1180,13 @@
       <c r="X3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="Y3" s="36"/>
+      <c r="Y3" s="43"/>
       <c r="Z3" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="AA3" s="38"/>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AA3" s="36"/>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1276,7 +1276,7 @@
         <v>0.42172276363636341</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>0.42172276363636363</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>0.26477524363636362</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>34</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>0.26477524363636368</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>32</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>0.26477524363636368</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>27</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>1.0029866036363635</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -1808,7 +1808,7 @@
         <v>0.51477524363636351</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>3.6717227636363634</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>56</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>1.0029866036363635</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -2082,7 +2082,7 @@
         <v>0.26477524363636362</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>1.0029866036363635</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>28</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>1.0029866036363635</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>0.26477524363636362</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>29</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>0.53214404363636381</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>52</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>0.53214404363636336</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>24</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>0.26477524363636368</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>14</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>0.51477524363636362</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>22</v>
       </c>
@@ -2814,7 +2814,7 @@
         <v>0.42172276363636363</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>26</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>0.26477524363636362</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>9</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>0.53214404363636381</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>16</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>0.26477524363636362</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>18</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>1.0029866036363635</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>20</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>0.53214404363636358</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>17</v>
       </c>
@@ -3370,7 +3370,7 @@
         <v>1.0029866036363635</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>10</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>1.5321440436363638</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>53</v>
       </c>
@@ -3550,7 +3550,7 @@
         <v>0.26477524363636357</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>30</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>0.42172276363636341</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>23</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>0.26477524363636357</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>36</v>
       </c>
@@ -3812,7 +3812,7 @@
         <v>0.26477524363636357</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>31</v>
       </c>
@@ -3902,7 +3902,7 @@
         <v>0.42172276363636363</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>37</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>0.26477524363636362</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>15</v>
       </c>
@@ -4074,7 +4074,7 @@
         <v>0.26477524363636357</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>19</v>
       </c>
@@ -4168,7 +4168,7 @@
         <v>0.53214404363636358</v>
       </c>
     </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
       <c r="AA37" s="1"/>
@@ -4178,13 +4178,6 @@
     <sortCondition ref="A3:A35"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
     <mergeCell ref="Y2:Y3"/>
     <mergeCell ref="AA2:AA3"/>
     <mergeCell ref="S2:U2"/>
@@ -4194,6 +4187,13 @@
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="M2:O2"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:AA36">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
@@ -4208,14 +4208,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>65</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>66</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>67</v>
       </c>
@@ -4266,7 +4266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>96</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>97</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>68</v>
       </c>
@@ -4317,9 +4317,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B7" s="34">
         <v>0.32078894883401449</v>
@@ -4334,7 +4334,7 @@
         <v>1.7643392185870794</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>69</v>
       </c>
@@ -4351,7 +4351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>94</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>70</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>1.4859070670060452</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>71</v>
       </c>
@@ -4402,7 +4402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>72</v>
       </c>
@@ -4419,7 +4419,7 @@
         <v>1.4868532033110473</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>73</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>2.1452484665135505</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>74</v>
       </c>
@@ -4453,7 +4453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>75</v>
       </c>
@@ -4470,7 +4470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>76</v>
       </c>
@@ -4487,7 +4487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>77</v>
       </c>
@@ -4504,7 +4504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>78</v>
       </c>
@@ -4521,7 +4521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>79</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>80</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>81</v>
       </c>
@@ -4572,7 +4572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>95</v>
       </c>
@@ -4606,7 +4606,7 @@
         <v>1.5235556475424097</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>83</v>
       </c>
@@ -4623,7 +4623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>84</v>
       </c>
@@ -4640,7 +4640,7 @@
         <v>1.4461826728736582</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>85</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="33" t="s">
         <v>86</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="33" t="s">
         <v>93</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="33" t="s">
         <v>87</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>88</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>89</v>
       </c>
@@ -4742,7 +4742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>90</v>
       </c>
@@ -4759,7 +4759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>91</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="33" t="s">
         <v>92</v>
       </c>
@@ -4793,9 +4793,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B35" s="34">
         <v>1</v>
@@ -4810,9 +4810,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B36" s="34">
         <v>1</v>
@@ -4827,9 +4827,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B37" s="34">
         <v>1</v>
@@ -4844,9 +4844,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B38" s="34">
         <v>1</v>
@@ -4861,9 +4861,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B39" s="34">
         <v>1</v>
@@ -4878,9 +4878,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B40" s="34">
         <v>1</v>
@@ -4912,28 +4912,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="13.453125" defaultRowHeight="23.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.42578125" defaultRowHeight="23.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.453125" style="26"/>
-    <col min="2" max="2" width="8.26953125" style="27" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" style="26"/>
-    <col min="4" max="4" width="9.7265625" style="27" customWidth="1"/>
-    <col min="5" max="5" width="14.26953125" style="26" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" style="26"/>
+    <col min="2" max="2" width="8.28515625" style="27" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" style="26"/>
+    <col min="4" max="4" width="9.7109375" style="27" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" style="26" customWidth="1"/>
     <col min="6" max="6" width="9" style="27" customWidth="1"/>
-    <col min="7" max="7" width="13.453125" style="28"/>
-    <col min="8" max="8" width="6.54296875" style="26" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" style="28"/>
-    <col min="10" max="10" width="6.7265625" style="27" customWidth="1"/>
-    <col min="11" max="11" width="11.453125" style="28" customWidth="1"/>
-    <col min="12" max="12" width="7.7265625" style="26" customWidth="1"/>
-    <col min="13" max="13" width="13.453125" style="28"/>
-    <col min="14" max="14" width="10.54296875" style="27" customWidth="1"/>
-    <col min="15" max="15" width="13.453125" style="28"/>
-    <col min="16" max="16" width="8.453125" style="27" customWidth="1"/>
-    <col min="17" max="16384" width="13.453125" style="26"/>
+    <col min="7" max="7" width="13.42578125" style="28"/>
+    <col min="8" max="8" width="6.5703125" style="26" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" style="28"/>
+    <col min="10" max="10" width="6.7109375" style="27" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" style="28" customWidth="1"/>
+    <col min="12" max="12" width="7.7109375" style="26" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" style="28"/>
+    <col min="14" max="14" width="10.5703125" style="27" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" style="28"/>
+    <col min="16" max="16" width="8.42578125" style="27" customWidth="1"/>
+    <col min="17" max="16384" width="13.42578125" style="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>57</v>
       </c>
@@ -4983,7 +4983,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
         <v>57</v>
       </c>
@@ -5027,7 +5027,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
         <v>57</v>
       </c>
@@ -5071,7 +5071,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>57</v>
       </c>
@@ -5115,7 +5115,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>57</v>
       </c>
@@ -5159,7 +5159,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>57</v>
       </c>
@@ -5203,7 +5203,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>57</v>
       </c>
@@ -5247,7 +5247,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>57</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>57</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
         <v>57</v>
       </c>
@@ -5379,7 +5379,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
         <v>57</v>
       </c>
@@ -5423,7 +5423,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
         <v>57</v>
       </c>
@@ -5467,7 +5467,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
         <v>57</v>
       </c>
@@ -5511,7 +5511,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>57</v>
       </c>
@@ -5555,7 +5555,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
         <v>57</v>
       </c>
@@ -5599,7 +5599,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
         <v>57</v>
       </c>
@@ -5643,7 +5643,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>57</v>
       </c>
@@ -5687,7 +5687,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
         <v>57</v>
       </c>
@@ -5731,7 +5731,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
         <v>57</v>
       </c>
@@ -5775,7 +5775,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
         <v>57</v>
       </c>
@@ -5819,7 +5819,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
         <v>57</v>
       </c>
@@ -5863,7 +5863,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
         <v>57</v>
       </c>
@@ -5907,7 +5907,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>57</v>
       </c>
@@ -5951,37 +5951,37 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="25" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="29" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="32" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="33" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="34" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="35" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="36" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="37" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="38" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="39" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="40" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="41" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="42" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="43" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="44" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="45" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="46" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="47" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="48" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="49" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="50" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="51" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="52" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="53" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="54" ht="30" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5991,14 +5991,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>4</v>
       </c>
@@ -6015,7 +6015,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="29" t="s">
         <v>11</v>
       </c>
@@ -6024,7 +6024,7 @@
       <c r="D2" s="30"/>
       <c r="E2" s="30"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
         <v>12</v>
       </c>
@@ -6033,7 +6033,7 @@
       <c r="D3" s="30"/>
       <c r="E3" s="30"/>
     </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
         <v>33</v>
       </c>
@@ -6042,7 +6042,7 @@
       <c r="D4" s="30"/>
       <c r="E4" s="30"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
         <v>34</v>
       </c>
@@ -6051,7 +6051,7 @@
       <c r="D5" s="30"/>
       <c r="E5" s="30"/>
     </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>32</v>
       </c>
@@ -6060,7 +6060,7 @@
       <c r="D6" s="30"/>
       <c r="E6" s="30"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
         <v>27</v>
       </c>
@@ -6069,7 +6069,7 @@
       <c r="D7" s="30"/>
       <c r="E7" s="30"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
         <v>13</v>
       </c>
@@ -6078,7 +6078,7 @@
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
         <v>21</v>
       </c>
@@ -6087,7 +6087,7 @@
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
         <v>56</v>
       </c>
@@ -6096,7 +6096,7 @@
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
         <v>25</v>
       </c>
@@ -6105,7 +6105,7 @@
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>8</v>
       </c>
@@ -6114,7 +6114,7 @@
       <c r="D12" s="30"/>
       <c r="E12" s="30"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
         <v>28</v>
       </c>
@@ -6123,7 +6123,7 @@
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
         <v>35</v>
       </c>
@@ -6132,7 +6132,7 @@
       <c r="D14" s="30"/>
       <c r="E14" s="30"/>
     </row>
-    <row r="15" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>29</v>
       </c>
@@ -6141,7 +6141,7 @@
       <c r="D15" s="30"/>
       <c r="E15" s="30"/>
     </row>
-    <row r="16" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
         <v>52</v>
       </c>
@@ -6150,7 +6150,7 @@
       <c r="D16" s="30"/>
       <c r="E16" s="30"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
         <v>24</v>
       </c>
@@ -6159,7 +6159,7 @@
       <c r="D17" s="30"/>
       <c r="E17" s="30"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>14</v>
       </c>
@@ -6168,7 +6168,7 @@
       <c r="D18" s="30"/>
       <c r="E18" s="30"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
         <v>22</v>
       </c>
@@ -6177,7 +6177,7 @@
       <c r="D19" s="30"/>
       <c r="E19" s="30"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
         <v>26</v>
       </c>
@@ -6186,7 +6186,7 @@
       <c r="D20" s="30"/>
       <c r="E20" s="30"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
         <v>9</v>
       </c>
@@ -6195,7 +6195,7 @@
       <c r="D21" s="30"/>
       <c r="E21" s="30"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
         <v>16</v>
       </c>
@@ -6204,7 +6204,7 @@
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
         <v>18</v>
       </c>
@@ -6213,7 +6213,7 @@
       <c r="D23" s="30"/>
       <c r="E23" s="30"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
         <v>20</v>
       </c>
@@ -6222,7 +6222,7 @@
       <c r="D24" s="30"/>
       <c r="E24" s="30"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
         <v>17</v>
       </c>
@@ -6231,7 +6231,7 @@
       <c r="D25" s="30"/>
       <c r="E25" s="30"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
         <v>10</v>
       </c>
@@ -6240,7 +6240,7 @@
       <c r="D26" s="30"/>
       <c r="E26" s="30"/>
     </row>
-    <row r="27" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="29" t="s">
         <v>30</v>
       </c>
@@ -6249,7 +6249,7 @@
       <c r="D27" s="30"/>
       <c r="E27" s="30"/>
     </row>
-    <row r="28" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
         <v>23</v>
       </c>
@@ -6258,7 +6258,7 @@
       <c r="D28" s="30"/>
       <c r="E28" s="30"/>
     </row>
-    <row r="29" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
         <v>36</v>
       </c>
@@ -6267,7 +6267,7 @@
       <c r="D29" s="30"/>
       <c r="E29" s="30"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="31" t="s">
         <v>31</v>
       </c>
@@ -6276,7 +6276,7 @@
       <c r="D30" s="30"/>
       <c r="E30" s="30"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="31" t="s">
         <v>37</v>
       </c>
@@ -6285,7 +6285,7 @@
       <c r="D31" s="30"/>
       <c r="E31" s="30"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
         <v>15</v>
       </c>
@@ -6294,7 +6294,7 @@
       <c r="D32" s="30"/>
       <c r="E32" s="30"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="31" t="s">
         <v>19</v>
       </c>
@@ -6303,7 +6303,7 @@
       <c r="D33" s="30"/>
       <c r="E33" s="30"/>
     </row>
-    <row r="34" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="29" t="s">
         <v>53</v>
       </c>

</xml_diff>